<commit_message>
docs: actualizar entregables hito 2
</commit_message>
<xml_diff>
--- a/docs/05_cronograma.xlsx
+++ b/docs/05_cronograma.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5E1F95-5C78-47C5-9150-AF883F186278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC08B00-E271-46FB-AFF1-68658CC31F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="61">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -135,9 +135,6 @@
     <t>Tarea 5</t>
   </si>
   <si>
-    <t>Título de la fase 2</t>
-  </si>
-  <si>
     <t>Título de la fase 3</t>
   </si>
   <si>
@@ -241,6 +238,30 @@
   </si>
   <si>
     <t>Adriana Tapia - Gerardo Ramos</t>
+  </si>
+  <si>
+    <t>Implementación de entidades</t>
+  </si>
+  <si>
+    <t>Creación de repositorios</t>
+  </si>
+  <si>
+    <t>Servicios y controllers</t>
+  </si>
+  <si>
+    <t>Seguridad</t>
+  </si>
+  <si>
+    <t>Documentación y PPT</t>
+  </si>
+  <si>
+    <t>Recolección de evidencias</t>
+  </si>
+  <si>
+    <t>Uso de herramienta de gestión</t>
+  </si>
+  <si>
+    <t>Avance de proyecto 2</t>
   </si>
 </sst>
 </file>
@@ -1050,7 +1071,7 @@
     <xf numFmtId="0" fontId="9" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1313,9 +1334,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="3" xfId="9">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="11" applyFont="1" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1937,22 +1955,22 @@
     </row>
     <row r="4" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A4" s="39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="35" customFormat="1" ht="215.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
@@ -1995,11 +2013,11 @@
     <tabColor rgb="FFF17604"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BL41"/>
+  <dimension ref="A1:BL43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="45" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
     <col min="3" max="3" width="30.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.7109375" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" style="5" customWidth="1"/>
@@ -2015,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="49" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
@@ -2036,10 +2054,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="51" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="88" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D3" s="89"/>
       <c r="E3" s="93">
@@ -2052,15 +2070,15 @@
         <v>3</v>
       </c>
       <c r="C4" s="88" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" s="89"/>
       <c r="E4" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4" s="90">
         <f>I5</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="J4" s="91"/>
       <c r="K4" s="91"/>
@@ -2070,7 +2088,7 @@
       <c r="O4" s="92"/>
       <c r="P4" s="90">
         <f>P5</f>
-        <v>46125</v>
+        <v>46146</v>
       </c>
       <c r="Q4" s="91"/>
       <c r="R4" s="91"/>
@@ -2080,7 +2098,7 @@
       <c r="V4" s="92"/>
       <c r="W4" s="90">
         <f>W5</f>
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="X4" s="91"/>
       <c r="Y4" s="91"/>
@@ -2090,7 +2108,7 @@
       <c r="AC4" s="92"/>
       <c r="AD4" s="90">
         <f>AD5</f>
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="AE4" s="91"/>
       <c r="AF4" s="91"/>
@@ -2100,7 +2118,7 @@
       <c r="AJ4" s="92"/>
       <c r="AK4" s="90">
         <f>AK5</f>
-        <v>46146</v>
+        <v>46167</v>
       </c>
       <c r="AL4" s="91"/>
       <c r="AM4" s="91"/>
@@ -2110,7 +2128,7 @@
       <c r="AQ4" s="92"/>
       <c r="AR4" s="90">
         <f>AR5</f>
-        <v>46153</v>
+        <v>46174</v>
       </c>
       <c r="AS4" s="91"/>
       <c r="AT4" s="91"/>
@@ -2120,7 +2138,7 @@
       <c r="AX4" s="92"/>
       <c r="AY4" s="90">
         <f>AY5</f>
-        <v>46160</v>
+        <v>46181</v>
       </c>
       <c r="AZ4" s="91"/>
       <c r="BA4" s="91"/>
@@ -2130,7 +2148,7 @@
       <c r="BE4" s="92"/>
       <c r="BF4" s="90">
         <f>BF5</f>
-        <v>46167</v>
+        <v>46188</v>
       </c>
       <c r="BG4" s="91"/>
       <c r="BH4" s="91"/>
@@ -2151,227 +2169,227 @@
       <c r="G5" s="66"/>
       <c r="I5" s="81">
         <f>Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
-        <v>46118</v>
+        <v>46139</v>
       </c>
       <c r="J5" s="82">
         <f>I5+1</f>
-        <v>46119</v>
+        <v>46140</v>
       </c>
       <c r="K5" s="82">
         <f t="shared" ref="K5:AX5" si="0">J5+1</f>
-        <v>46120</v>
+        <v>46141</v>
       </c>
       <c r="L5" s="82">
         <f t="shared" si="0"/>
-        <v>46121</v>
+        <v>46142</v>
       </c>
       <c r="M5" s="82">
         <f t="shared" si="0"/>
-        <v>46122</v>
+        <v>46143</v>
       </c>
       <c r="N5" s="82">
         <f t="shared" si="0"/>
-        <v>46123</v>
+        <v>46144</v>
       </c>
       <c r="O5" s="83">
         <f t="shared" si="0"/>
-        <v>46124</v>
+        <v>46145</v>
       </c>
       <c r="P5" s="81">
         <f>O5+1</f>
-        <v>46125</v>
+        <v>46146</v>
       </c>
       <c r="Q5" s="82">
         <f>P5+1</f>
-        <v>46126</v>
+        <v>46147</v>
       </c>
       <c r="R5" s="82">
         <f t="shared" si="0"/>
-        <v>46127</v>
+        <v>46148</v>
       </c>
       <c r="S5" s="82">
         <f t="shared" si="0"/>
-        <v>46128</v>
+        <v>46149</v>
       </c>
       <c r="T5" s="82">
         <f t="shared" si="0"/>
-        <v>46129</v>
+        <v>46150</v>
       </c>
       <c r="U5" s="82">
         <f t="shared" si="0"/>
-        <v>46130</v>
+        <v>46151</v>
       </c>
       <c r="V5" s="83">
         <f t="shared" si="0"/>
-        <v>46131</v>
+        <v>46152</v>
       </c>
       <c r="W5" s="81">
         <f>V5+1</f>
-        <v>46132</v>
+        <v>46153</v>
       </c>
       <c r="X5" s="82">
         <f>W5+1</f>
-        <v>46133</v>
+        <v>46154</v>
       </c>
       <c r="Y5" s="82">
         <f t="shared" si="0"/>
-        <v>46134</v>
+        <v>46155</v>
       </c>
       <c r="Z5" s="82">
         <f t="shared" si="0"/>
-        <v>46135</v>
+        <v>46156</v>
       </c>
       <c r="AA5" s="82">
         <f t="shared" si="0"/>
-        <v>46136</v>
+        <v>46157</v>
       </c>
       <c r="AB5" s="82">
         <f t="shared" si="0"/>
-        <v>46137</v>
+        <v>46158</v>
       </c>
       <c r="AC5" s="83">
         <f t="shared" si="0"/>
-        <v>46138</v>
+        <v>46159</v>
       </c>
       <c r="AD5" s="81">
         <f>AC5+1</f>
-        <v>46139</v>
+        <v>46160</v>
       </c>
       <c r="AE5" s="82">
         <f>AD5+1</f>
-        <v>46140</v>
+        <v>46161</v>
       </c>
       <c r="AF5" s="82">
         <f t="shared" si="0"/>
-        <v>46141</v>
+        <v>46162</v>
       </c>
       <c r="AG5" s="82">
         <f t="shared" si="0"/>
-        <v>46142</v>
+        <v>46163</v>
       </c>
       <c r="AH5" s="82">
         <f t="shared" si="0"/>
-        <v>46143</v>
+        <v>46164</v>
       </c>
       <c r="AI5" s="82">
         <f t="shared" si="0"/>
-        <v>46144</v>
+        <v>46165</v>
       </c>
       <c r="AJ5" s="83">
         <f t="shared" si="0"/>
-        <v>46145</v>
+        <v>46166</v>
       </c>
       <c r="AK5" s="81">
         <f>AJ5+1</f>
-        <v>46146</v>
+        <v>46167</v>
       </c>
       <c r="AL5" s="82">
         <f>AK5+1</f>
-        <v>46147</v>
+        <v>46168</v>
       </c>
       <c r="AM5" s="82">
         <f t="shared" si="0"/>
-        <v>46148</v>
+        <v>46169</v>
       </c>
       <c r="AN5" s="82">
         <f t="shared" si="0"/>
-        <v>46149</v>
+        <v>46170</v>
       </c>
       <c r="AO5" s="82">
         <f t="shared" si="0"/>
-        <v>46150</v>
+        <v>46171</v>
       </c>
       <c r="AP5" s="82">
         <f t="shared" si="0"/>
-        <v>46151</v>
+        <v>46172</v>
       </c>
       <c r="AQ5" s="83">
         <f t="shared" si="0"/>
-        <v>46152</v>
+        <v>46173</v>
       </c>
       <c r="AR5" s="81">
         <f>AQ5+1</f>
-        <v>46153</v>
+        <v>46174</v>
       </c>
       <c r="AS5" s="82">
         <f>AR5+1</f>
-        <v>46154</v>
+        <v>46175</v>
       </c>
       <c r="AT5" s="82">
         <f t="shared" si="0"/>
-        <v>46155</v>
+        <v>46176</v>
       </c>
       <c r="AU5" s="82">
         <f t="shared" si="0"/>
-        <v>46156</v>
+        <v>46177</v>
       </c>
       <c r="AV5" s="82">
         <f t="shared" si="0"/>
-        <v>46157</v>
+        <v>46178</v>
       </c>
       <c r="AW5" s="82">
         <f t="shared" si="0"/>
-        <v>46158</v>
+        <v>46179</v>
       </c>
       <c r="AX5" s="83">
         <f t="shared" si="0"/>
-        <v>46159</v>
+        <v>46180</v>
       </c>
       <c r="AY5" s="81">
         <f>AX5+1</f>
-        <v>46160</v>
+        <v>46181</v>
       </c>
       <c r="AZ5" s="82">
         <f>AY5+1</f>
-        <v>46161</v>
+        <v>46182</v>
       </c>
       <c r="BA5" s="82">
         <f t="shared" ref="BA5:BE5" si="1">AZ5+1</f>
-        <v>46162</v>
+        <v>46183</v>
       </c>
       <c r="BB5" s="82">
         <f t="shared" si="1"/>
-        <v>46163</v>
+        <v>46184</v>
       </c>
       <c r="BC5" s="82">
         <f t="shared" si="1"/>
-        <v>46164</v>
+        <v>46185</v>
       </c>
       <c r="BD5" s="82">
         <f t="shared" si="1"/>
-        <v>46165</v>
+        <v>46186</v>
       </c>
       <c r="BE5" s="83">
         <f t="shared" si="1"/>
-        <v>46166</v>
+        <v>46187</v>
       </c>
       <c r="BF5" s="81">
         <f>BE5+1</f>
-        <v>46167</v>
+        <v>46188</v>
       </c>
       <c r="BG5" s="82">
         <f>BF5+1</f>
-        <v>46168</v>
+        <v>46189</v>
       </c>
       <c r="BH5" s="82">
         <f t="shared" ref="BH5:BL5" si="2">BG5+1</f>
-        <v>46169</v>
+        <v>46190</v>
       </c>
       <c r="BI5" s="82">
         <f t="shared" si="2"/>
-        <v>46170</v>
+        <v>46191</v>
       </c>
       <c r="BJ5" s="82">
         <f t="shared" si="2"/>
-        <v>46171</v>
+        <v>46192</v>
       </c>
       <c r="BK5" s="82">
         <f t="shared" si="2"/>
-        <v>46172</v>
+        <v>46193</v>
       </c>
       <c r="BL5" s="83">
         <f t="shared" si="2"/>
-        <v>46173</v>
+        <v>46194</v>
       </c>
     </row>
     <row r="6" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2382,20 +2400,20 @@
         <v>14</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>28</v>
-      </c>
       <c r="F6" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I6" s="10" t="str">
         <f t="shared" ref="I6" si="3">LEFT(TEXT(I5,"ddd"),1)</f>
@@ -2694,7 +2712,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="52"/>
       <c r="D8" s="16"/>
@@ -2702,7 +2720,7 @@
       <c r="F8" s="71"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14" t="str">
-        <f t="shared" ref="H8:H38" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H8:H40" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="31"/>
@@ -2767,10 +2785,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="53" t="s">
         <v>40</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>41</v>
       </c>
       <c r="D9" s="17">
         <v>1</v>
@@ -2849,10 +2867,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="61" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" s="17">
         <v>1</v>
@@ -2928,10 +2946,10 @@
     <row r="11" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="45"/>
       <c r="B11" s="61" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" s="17">
         <v>1</v>
@@ -3007,10 +3025,10 @@
     <row r="12" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="45"/>
       <c r="B12" s="61" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="53" t="s">
         <v>43</v>
-      </c>
-      <c r="C12" s="53" t="s">
-        <v>44</v>
       </c>
       <c r="D12" s="17">
         <v>1</v>
@@ -3083,10 +3101,10 @@
     <row r="13" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="45"/>
       <c r="B13" s="61" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D13" s="17">
         <v>1</v>
@@ -3162,10 +3180,10 @@
     <row r="14" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="45"/>
       <c r="B14" s="61" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="53" t="s">
         <v>46</v>
-      </c>
-      <c r="C14" s="53" t="s">
-        <v>47</v>
       </c>
       <c r="D14" s="17">
         <v>1</v>
@@ -3238,10 +3256,10 @@
     <row r="15" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="45"/>
       <c r="B15" s="61" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="94" t="s">
-        <v>53</v>
+        <v>48</v>
+      </c>
+      <c r="C15" s="53" t="s">
+        <v>52</v>
       </c>
       <c r="D15" s="17">
         <v>1</v>
@@ -3317,10 +3335,10 @@
     <row r="16" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="45"/>
       <c r="B16" s="61" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="94" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="C16" s="53" t="s">
+        <v>47</v>
       </c>
       <c r="D16" s="17">
         <v>1</v>
@@ -3393,10 +3411,10 @@
     <row r="17" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45"/>
       <c r="B17" s="61" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="94" t="s">
-        <v>53</v>
+        <v>50</v>
+      </c>
+      <c r="C17" s="53" t="s">
+        <v>52</v>
       </c>
       <c r="D17" s="17">
         <v>1</v>
@@ -3469,10 +3487,10 @@
     <row r="18" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="45"/>
       <c r="B18" s="61" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="94" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="C18" s="53" t="s">
+        <v>43</v>
       </c>
       <c r="D18" s="17">
         <v>1</v>
@@ -3547,7 +3565,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="C19" s="54"/>
       <c r="D19" s="19"/>
@@ -3618,24 +3636,24 @@
     <row r="20" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="46"/>
       <c r="B20" s="62" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="55"/>
+        <v>53</v>
+      </c>
+      <c r="C20" s="55" t="s">
+        <v>40</v>
+      </c>
       <c r="D20" s="20">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E20" s="85">
-        <f>E15+1</f>
-        <v>46136</v>
+        <v>46143</v>
       </c>
       <c r="F20" s="85">
-        <f>E20+4</f>
-        <v>46140</v>
+        <v>46145</v>
       </c>
       <c r="G20" s="14"/>
       <c r="H20" s="14">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31"/>
@@ -3697,24 +3715,25 @@
     <row r="21" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="45"/>
       <c r="B21" s="62" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="55"/>
+        <v>54</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>46</v>
+      </c>
       <c r="D21" s="20">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E21" s="85">
         <f>E20+2</f>
-        <v>46138</v>
+        <v>46145</v>
       </c>
       <c r="F21" s="85">
-        <f>E21+5</f>
-        <v>46143</v>
+        <v>46147</v>
       </c>
       <c r="G21" s="14"/>
       <c r="H21" s="14">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I21" s="31"/>
       <c r="J21" s="31"/>
@@ -3776,17 +3795,19 @@
     <row r="22" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="45"/>
       <c r="B22" s="62" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="55"/>
-      <c r="D22" s="20"/>
+        <v>55</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="20">
+        <v>1</v>
+      </c>
       <c r="E22" s="85">
-        <f>F21</f>
-        <v>46143</v>
+        <v>46148</v>
       </c>
       <c r="F22" s="85">
-        <f>E22+3</f>
-        <v>46146</v>
+        <v>46151</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14">
@@ -3853,22 +3874,24 @@
     <row r="23" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="45"/>
       <c r="B23" s="62" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="55"/>
-      <c r="D23" s="20"/>
+        <v>56</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="20">
+        <v>1</v>
+      </c>
       <c r="E23" s="85">
-        <f>E22</f>
-        <v>46143</v>
+        <v>46152</v>
       </c>
       <c r="F23" s="85">
-        <f>E23+2</f>
-        <v>46145</v>
+        <v>46156</v>
       </c>
       <c r="G23" s="14"/>
       <c r="H23" s="14">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -3930,23 +3953,22 @@
     <row r="24" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="45"/>
       <c r="B24" s="62" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="55"/>
-      <c r="D24" s="20"/>
+        <v>57</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="20">
+        <v>0.9</v>
+      </c>
       <c r="E24" s="85">
-        <f>E23</f>
-        <v>46143</v>
+        <v>46154</v>
       </c>
       <c r="F24" s="85">
-        <f>E24+3</f>
-        <v>46146</v>
+        <v>46158</v>
       </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
+      <c r="H24" s="14"/>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
       <c r="K24" s="31"/>
@@ -3963,7 +3985,7 @@
       <c r="V24" s="31"/>
       <c r="W24" s="31"/>
       <c r="X24" s="31"/>
-      <c r="Y24" s="31"/>
+      <c r="Y24" s="32"/>
       <c r="Z24" s="31"/>
       <c r="AA24" s="31"/>
       <c r="AB24" s="31"/>
@@ -4005,20 +4027,26 @@
       <c r="BL24" s="31"/>
     </row>
     <row r="25" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="56"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="74"/>
-      <c r="F25" s="75"/>
+      <c r="A25" s="45"/>
+      <c r="B25" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="20">
+        <v>1</v>
+      </c>
+      <c r="E25" s="85">
+        <v>46158</v>
+      </c>
+      <c r="F25" s="85">
+        <v>46163</v>
+      </c>
       <c r="G25" s="14"/>
-      <c r="H25" s="14" t="str">
+      <c r="H25" s="14">
         <f t="shared" si="6"/>
-        <v/>
+        <v>6</v>
       </c>
       <c r="I25" s="31"/>
       <c r="J25" s="31"/>
@@ -4079,24 +4107,23 @@
     </row>
     <row r="26" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="45"/>
-      <c r="B26" s="63" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="57"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="76">
-        <f>E9+15</f>
-        <v>46137</v>
-      </c>
-      <c r="F26" s="76">
-        <f>E26+5</f>
-        <v>46142</v>
+      <c r="B26" s="62" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="20">
+        <v>1</v>
+      </c>
+      <c r="E26" s="85">
+        <v>46164</v>
+      </c>
+      <c r="F26" s="85">
+        <v>46167</v>
       </c>
       <c r="G26" s="14"/>
-      <c r="H26" s="14">
-        <f t="shared" si="6"/>
-        <v>6</v>
-      </c>
+      <c r="H26" s="14"/>
       <c r="I26" s="31"/>
       <c r="J26" s="31"/>
       <c r="K26" s="31"/>
@@ -4155,24 +4182,20 @@
       <c r="BL26" s="31"/>
     </row>
     <row r="27" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="45"/>
-      <c r="B27" s="63" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="57"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="76">
-        <f>F26+1</f>
-        <v>46143</v>
-      </c>
-      <c r="F27" s="76">
-        <f>E27+4</f>
-        <v>46147</v>
-      </c>
+      <c r="A27" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="56"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="74"/>
+      <c r="F27" s="75"/>
       <c r="G27" s="14"/>
-      <c r="H27" s="14">
+      <c r="H27" s="14" t="str">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v/>
       </c>
       <c r="I27" s="31"/>
       <c r="J27" s="31"/>
@@ -4234,17 +4257,17 @@
     <row r="28" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="45"/>
       <c r="B28" s="63" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C28" s="57"/>
       <c r="D28" s="23"/>
       <c r="E28" s="76">
-        <f>E27+5</f>
-        <v>46148</v>
+        <f>E9+15</f>
+        <v>46137</v>
       </c>
       <c r="F28" s="76">
         <f>E28+5</f>
-        <v>46153</v>
+        <v>46142</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14">
@@ -4311,17 +4334,17 @@
     <row r="29" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="45"/>
       <c r="B29" s="63" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C29" s="57"/>
       <c r="D29" s="23"/>
       <c r="E29" s="76">
         <f>F28+1</f>
-        <v>46154</v>
+        <v>46143</v>
       </c>
       <c r="F29" s="76">
         <f>E29+4</f>
-        <v>46158</v>
+        <v>46147</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="14">
@@ -4388,22 +4411,22 @@
     <row r="30" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="45"/>
       <c r="B30" s="63" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C30" s="57"/>
       <c r="D30" s="23"/>
       <c r="E30" s="76">
-        <f>E28</f>
+        <f>E29+5</f>
         <v>46148</v>
       </c>
       <c r="F30" s="76">
-        <f>E30+4</f>
-        <v>46152</v>
+        <f>E30+5</f>
+        <v>46153</v>
       </c>
       <c r="G30" s="14"/>
       <c r="H30" s="14">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I30" s="31"/>
       <c r="J30" s="31"/>
@@ -4463,20 +4486,24 @@
       <c r="BL30" s="31"/>
     </row>
     <row r="31" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C31" s="58"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="77"/>
-      <c r="F31" s="78"/>
+      <c r="A31" s="45"/>
+      <c r="B31" s="63" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="57"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="76">
+        <f>F30+1</f>
+        <v>46154</v>
+      </c>
+      <c r="F31" s="76">
+        <f>E31+4</f>
+        <v>46158</v>
+      </c>
       <c r="G31" s="14"/>
-      <c r="H31" s="14" t="str">
+      <c r="H31" s="14">
         <f t="shared" si="6"/>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I31" s="31"/>
       <c r="J31" s="31"/>
@@ -4537,21 +4564,23 @@
     </row>
     <row r="32" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="45"/>
-      <c r="B32" s="64" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="86" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="86" t="s">
-        <v>29</v>
+      <c r="B32" s="63" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="57"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="76">
+        <f>E30</f>
+        <v>46148</v>
+      </c>
+      <c r="F32" s="76">
+        <f>E32+4</f>
+        <v>46152</v>
       </c>
       <c r="G32" s="14"/>
-      <c r="H32" s="14" t="e">
+      <c r="H32" s="14">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v>5</v>
       </c>
       <c r="I32" s="31"/>
       <c r="J32" s="31"/>
@@ -4611,22 +4640,20 @@
       <c r="BL32" s="31"/>
     </row>
     <row r="33" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="45"/>
-      <c r="B33" s="64" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" s="59"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="86" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" s="86" t="s">
-        <v>29</v>
-      </c>
+      <c r="A33" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="58"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="78"/>
       <c r="G33" s="14"/>
-      <c r="H33" s="14" t="e">
+      <c r="H33" s="14" t="str">
         <f t="shared" si="6"/>
-        <v>#VALUE!</v>
+        <v/>
       </c>
       <c r="I33" s="31"/>
       <c r="J33" s="31"/>
@@ -4688,15 +4715,15 @@
     <row r="34" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="45"/>
       <c r="B34" s="64" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C34" s="59"/>
       <c r="D34" s="26"/>
       <c r="E34" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F34" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G34" s="14"/>
       <c r="H34" s="14" t="e">
@@ -4763,15 +4790,15 @@
     <row r="35" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="45"/>
       <c r="B35" s="64" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C35" s="59"/>
       <c r="D35" s="26"/>
       <c r="E35" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F35" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="14" t="e">
@@ -4838,15 +4865,15 @@
     <row r="36" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="45"/>
       <c r="B36" s="64" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C36" s="59"/>
       <c r="D36" s="26"/>
       <c r="E36" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F36" s="86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="14" t="e">
@@ -4911,18 +4938,22 @@
       <c r="BL36" s="31"/>
     </row>
     <row r="37" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="B37" s="65"/>
-      <c r="C37" s="60"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="87"/>
-      <c r="F37" s="87"/>
+      <c r="A37" s="45"/>
+      <c r="B37" s="64" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="59"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="86" t="s">
+        <v>28</v>
+      </c>
       <c r="G37" s="14"/>
-      <c r="H37" s="14" t="str">
+      <c r="H37" s="14" t="e">
         <f t="shared" si="6"/>
-        <v/>
+        <v>#VALUE!</v>
       </c>
       <c r="I37" s="31"/>
       <c r="J37" s="31"/>
@@ -4982,87 +5013,233 @@
       <c r="BL37" s="31"/>
     </row>
     <row r="38" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C38" s="28"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="79"/>
-      <c r="F38" s="80"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30" t="str">
+      <c r="A38" s="45"/>
+      <c r="B38" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="59"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="F38" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14" t="e">
+        <f t="shared" si="6"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I38" s="31"/>
+      <c r="J38" s="31"/>
+      <c r="K38" s="31"/>
+      <c r="L38" s="31"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="31"/>
+      <c r="P38" s="31"/>
+      <c r="Q38" s="31"/>
+      <c r="R38" s="31"/>
+      <c r="S38" s="31"/>
+      <c r="T38" s="31"/>
+      <c r="U38" s="31"/>
+      <c r="V38" s="31"/>
+      <c r="W38" s="31"/>
+      <c r="X38" s="31"/>
+      <c r="Y38" s="31"/>
+      <c r="Z38" s="31"/>
+      <c r="AA38" s="31"/>
+      <c r="AB38" s="31"/>
+      <c r="AC38" s="31"/>
+      <c r="AD38" s="31"/>
+      <c r="AE38" s="31"/>
+      <c r="AF38" s="31"/>
+      <c r="AG38" s="31"/>
+      <c r="AH38" s="31"/>
+      <c r="AI38" s="31"/>
+      <c r="AJ38" s="31"/>
+      <c r="AK38" s="31"/>
+      <c r="AL38" s="31"/>
+      <c r="AM38" s="31"/>
+      <c r="AN38" s="31"/>
+      <c r="AO38" s="31"/>
+      <c r="AP38" s="31"/>
+      <c r="AQ38" s="31"/>
+      <c r="AR38" s="31"/>
+      <c r="AS38" s="31"/>
+      <c r="AT38" s="31"/>
+      <c r="AU38" s="31"/>
+      <c r="AV38" s="31"/>
+      <c r="AW38" s="31"/>
+      <c r="AX38" s="31"/>
+      <c r="AY38" s="31"/>
+      <c r="AZ38" s="31"/>
+      <c r="BA38" s="31"/>
+      <c r="BB38" s="31"/>
+      <c r="BC38" s="31"/>
+      <c r="BD38" s="31"/>
+      <c r="BE38" s="31"/>
+      <c r="BF38" s="31"/>
+      <c r="BG38" s="31"/>
+      <c r="BH38" s="31"/>
+      <c r="BI38" s="31"/>
+      <c r="BJ38" s="31"/>
+      <c r="BK38" s="31"/>
+      <c r="BL38" s="31"/>
+    </row>
+    <row r="39" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="65"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="87"/>
+      <c r="F39" s="87"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="I38" s="33"/>
-      <c r="J38" s="33"/>
-      <c r="K38" s="33"/>
-      <c r="L38" s="33"/>
-      <c r="M38" s="33"/>
-      <c r="N38" s="33"/>
-      <c r="O38" s="33"/>
-      <c r="P38" s="33"/>
-      <c r="Q38" s="33"/>
-      <c r="R38" s="33"/>
-      <c r="S38" s="33"/>
-      <c r="T38" s="33"/>
-      <c r="U38" s="33"/>
-      <c r="V38" s="33"/>
-      <c r="W38" s="33"/>
-      <c r="X38" s="33"/>
-      <c r="Y38" s="33"/>
-      <c r="Z38" s="33"/>
-      <c r="AA38" s="33"/>
-      <c r="AB38" s="33"/>
-      <c r="AC38" s="33"/>
-      <c r="AD38" s="33"/>
-      <c r="AE38" s="33"/>
-      <c r="AF38" s="33"/>
-      <c r="AG38" s="33"/>
-      <c r="AH38" s="33"/>
-      <c r="AI38" s="33"/>
-      <c r="AJ38" s="33"/>
-      <c r="AK38" s="33"/>
-      <c r="AL38" s="33"/>
-      <c r="AM38" s="33"/>
-      <c r="AN38" s="33"/>
-      <c r="AO38" s="33"/>
-      <c r="AP38" s="33"/>
-      <c r="AQ38" s="33"/>
-      <c r="AR38" s="33"/>
-      <c r="AS38" s="33"/>
-      <c r="AT38" s="33"/>
-      <c r="AU38" s="33"/>
-      <c r="AV38" s="33"/>
-      <c r="AW38" s="33"/>
-      <c r="AX38" s="33"/>
-      <c r="AY38" s="33"/>
-      <c r="AZ38" s="33"/>
-      <c r="BA38" s="33"/>
-      <c r="BB38" s="33"/>
-      <c r="BC38" s="33"/>
-      <c r="BD38" s="33"/>
-      <c r="BE38" s="33"/>
-      <c r="BF38" s="33"/>
-      <c r="BG38" s="33"/>
-      <c r="BH38" s="33"/>
-      <c r="BI38" s="33"/>
-      <c r="BJ38" s="33"/>
-      <c r="BK38" s="33"/>
-      <c r="BL38" s="33"/>
-    </row>
-    <row r="39" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G39" s="6"/>
-    </row>
-    <row r="40" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="11"/>
-      <c r="F40" s="47"/>
+      <c r="I39" s="31"/>
+      <c r="J39" s="31"/>
+      <c r="K39" s="31"/>
+      <c r="L39" s="31"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="31"/>
+      <c r="P39" s="31"/>
+      <c r="Q39" s="31"/>
+      <c r="R39" s="31"/>
+      <c r="S39" s="31"/>
+      <c r="T39" s="31"/>
+      <c r="U39" s="31"/>
+      <c r="V39" s="31"/>
+      <c r="W39" s="31"/>
+      <c r="X39" s="31"/>
+      <c r="Y39" s="31"/>
+      <c r="Z39" s="31"/>
+      <c r="AA39" s="31"/>
+      <c r="AB39" s="31"/>
+      <c r="AC39" s="31"/>
+      <c r="AD39" s="31"/>
+      <c r="AE39" s="31"/>
+      <c r="AF39" s="31"/>
+      <c r="AG39" s="31"/>
+      <c r="AH39" s="31"/>
+      <c r="AI39" s="31"/>
+      <c r="AJ39" s="31"/>
+      <c r="AK39" s="31"/>
+      <c r="AL39" s="31"/>
+      <c r="AM39" s="31"/>
+      <c r="AN39" s="31"/>
+      <c r="AO39" s="31"/>
+      <c r="AP39" s="31"/>
+      <c r="AQ39" s="31"/>
+      <c r="AR39" s="31"/>
+      <c r="AS39" s="31"/>
+      <c r="AT39" s="31"/>
+      <c r="AU39" s="31"/>
+      <c r="AV39" s="31"/>
+      <c r="AW39" s="31"/>
+      <c r="AX39" s="31"/>
+      <c r="AY39" s="31"/>
+      <c r="AZ39" s="31"/>
+      <c r="BA39" s="31"/>
+      <c r="BB39" s="31"/>
+      <c r="BC39" s="31"/>
+      <c r="BD39" s="31"/>
+      <c r="BE39" s="31"/>
+      <c r="BF39" s="31"/>
+      <c r="BG39" s="31"/>
+      <c r="BH39" s="31"/>
+      <c r="BI39" s="31"/>
+      <c r="BJ39" s="31"/>
+      <c r="BK39" s="31"/>
+      <c r="BL39" s="31"/>
+    </row>
+    <row r="40" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C40" s="28"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="79"/>
+      <c r="F40" s="80"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="30" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="I40" s="33"/>
+      <c r="J40" s="33"/>
+      <c r="K40" s="33"/>
+      <c r="L40" s="33"/>
+      <c r="M40" s="33"/>
+      <c r="N40" s="33"/>
+      <c r="O40" s="33"/>
+      <c r="P40" s="33"/>
+      <c r="Q40" s="33"/>
+      <c r="R40" s="33"/>
+      <c r="S40" s="33"/>
+      <c r="T40" s="33"/>
+      <c r="U40" s="33"/>
+      <c r="V40" s="33"/>
+      <c r="W40" s="33"/>
+      <c r="X40" s="33"/>
+      <c r="Y40" s="33"/>
+      <c r="Z40" s="33"/>
+      <c r="AA40" s="33"/>
+      <c r="AB40" s="33"/>
+      <c r="AC40" s="33"/>
+      <c r="AD40" s="33"/>
+      <c r="AE40" s="33"/>
+      <c r="AF40" s="33"/>
+      <c r="AG40" s="33"/>
+      <c r="AH40" s="33"/>
+      <c r="AI40" s="33"/>
+      <c r="AJ40" s="33"/>
+      <c r="AK40" s="33"/>
+      <c r="AL40" s="33"/>
+      <c r="AM40" s="33"/>
+      <c r="AN40" s="33"/>
+      <c r="AO40" s="33"/>
+      <c r="AP40" s="33"/>
+      <c r="AQ40" s="33"/>
+      <c r="AR40" s="33"/>
+      <c r="AS40" s="33"/>
+      <c r="AT40" s="33"/>
+      <c r="AU40" s="33"/>
+      <c r="AV40" s="33"/>
+      <c r="AW40" s="33"/>
+      <c r="AX40" s="33"/>
+      <c r="AY40" s="33"/>
+      <c r="AZ40" s="33"/>
+      <c r="BA40" s="33"/>
+      <c r="BB40" s="33"/>
+      <c r="BC40" s="33"/>
+      <c r="BD40" s="33"/>
+      <c r="BE40" s="33"/>
+      <c r="BF40" s="33"/>
+      <c r="BG40" s="33"/>
+      <c r="BH40" s="33"/>
+      <c r="BI40" s="33"/>
+      <c r="BJ40" s="33"/>
+      <c r="BK40" s="33"/>
+      <c r="BL40" s="33"/>
     </row>
     <row r="41" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="12"/>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C42" s="11"/>
+      <c r="F42" s="47"/>
+    </row>
+    <row r="43" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C43" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -5078,7 +5255,7 @@
     <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
   </mergeCells>
-  <conditionalFormatting sqref="D7:D38">
+  <conditionalFormatting sqref="D7:D40">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5092,12 +5269,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:BL38">
+  <conditionalFormatting sqref="I5:BL40">
     <cfRule type="expression" dxfId="2" priority="33">
       <formula>AND(TODAY()&gt;=I$5,TODAY()&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:BL38">
+  <conditionalFormatting sqref="I7:BL40">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
@@ -5117,7 +5294,7 @@
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="F23 F27:F28 E28" formula="1"/>
+    <ignoredError sqref="F29:F30 E30" formula="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -5135,7 +5312,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D38</xm:sqref>
+          <xm:sqref>D7:D40</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5144,6 +5321,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5431,7 +5628,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -5440,27 +5637,19 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F80F839-78EF-4FF4-A673-3CC84279C232}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5481,22 +5670,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>